<commit_message>
Add Heritage format status columns to SWI register; mark 201-001 done
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Martabe tanpa SWI" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SWI vs Martabe'!$A$1:$E$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'SWI vs Martabe'!$A$1:$H$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -94,6 +94,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:H100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -467,6 +470,9 @@
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="95" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,6 +501,21 @@
           <t>Perbedaan SWI dengan data Martabe</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Format Heritage</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Tanggal konversi</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Catatan konversi</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -520,6 +541,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Dikonversi dari 304-008 heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-001.md</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -545,6 +581,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -570,6 +613,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
@@ -595,6 +645,13 @@
           <t>Martabe mengukur karbon yang terbawa ke launder (indikasi kehilangan karbon); SWI hanya mengukur larutan. Sumber Martabe tidak menyebut tujuan, volume sampler, suhu dan lama oven, sehingga rumus konsentrasi tidak ada. Bahaya Martabe: percikan slurry, sampler membentur kepala, titik jepit tutup titik sampling.</t>
         </is>
       </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
@@ -622,6 +679,13 @@
 2. Seluruhnya tambahan. Martabe memakai batas alarm HCN di bawah 10 ppm, SWI 5 ppm (SWI diterapkan). Angka plus-minus rentang di sumber tidak jelas.</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -647,6 +711,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -672,6 +743,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -697,6 +775,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -722,6 +807,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -747,6 +839,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -772,6 +871,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -797,6 +903,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n"/>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
@@ -826,6 +939,13 @@
 3. Seluruhnya tambahan. Sumber tidak memberi pH akhir pembilasan atau kekuatan asam, dan tidak menyebut risiko HCN dari asam pada sianida.</t>
         </is>
       </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -851,6 +971,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -876,6 +1003,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -901,6 +1035,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
@@ -926,6 +1067,13 @@
           <t>Tambahan; mendukung 204-010 (kekuatan larutan). Hazard Martabe: kontak flokulan, lantai licin, titik jepit valve, jangan sampling saat ada pengangkatan flokulan.</t>
         </is>
       </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -951,6 +1099,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n"/>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
@@ -976,6 +1131,13 @@
           <t>Martabe untuk filter air potabel, bukan discharge WTP berlisensi, sehingga hanya dijadikan referensi teknik; SWI tetap NOT FOR USE. 'SLS' dan paket assay tidak didefinisikan.</t>
         </is>
       </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
@@ -1005,6 +1167,13 @@
 3. Titik sampel berbeda (pipa drain pompa); perlu konfirmasi pipa itu membawa larutan encer. Titran H2SO4 (rasio 2:1) vs HCl (1:1).</t>
         </is>
       </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n"/>
+      <c r="H21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1030,6 +1199,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1057,6 +1233,13 @@
 2. Tambahan. Toleransi hanya lewat contoh (sekitar 0.2 pH) padahal batas keselamatan sianida pH di atas 10.5; buffer hanya 7 dan 10 (SWI 206-004 memakai 4, 7, 10).</t>
         </is>
       </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1082,6 +1265,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n"/>
+      <c r="H24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1107,6 +1297,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1132,6 +1329,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n"/>
+      <c r="H26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1157,6 +1361,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1182,6 +1393,13 @@
           <t>Martabe memakai komposit banyak cuplikan dan pembanding persen padatan di lab; SWI memakai cut berwaktu dan tonase. Prinsip sama (jangan disetel sendiri). Martabe meminta control room mematikan pompa barren dan sump (alasan tidak disebut; daftar milik Martabe); rumus persen padatan tidak ada.</t>
         </is>
       </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1207,6 +1425,13 @@
           <t>Martabe hanya teknik pengambilan sampel (tanpa analisis ukuran); SWI hanya prinsip. Ditulis untuk ball mill dan VertiMill; pabrik Anda memakai IsaMill. Titik jangkar harness dan fungsi saklar tidak dijelaskan.</t>
         </is>
       </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1232,6 +1457,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1257,6 +1489,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1282,6 +1521,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1307,6 +1553,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1332,6 +1585,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="n"/>
+      <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1357,6 +1617,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1382,6 +1649,13 @@
           <t>Martabe berbasis pengukuran celah dan umur screen, SWI berbasis kehilangan massa. Sumber menyebut bahaya tetapi tidak memberi kontrol. Perlu konfirmasi ada intertank screen dalam tangki dan batas 1.4 mm terhadap register aperture.</t>
         </is>
       </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -1407,6 +1681,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1432,6 +1713,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -1457,6 +1745,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -1482,6 +1777,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -1507,6 +1809,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -1532,6 +1841,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -1557,6 +1873,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -1582,6 +1905,13 @@
           <t>Martabe memverifikasi alat, bukan metode sampel. Tidak ada nilai penerimaan (teoretis sekitar 15.7 persen air). Moisture analyser tidak ada di daftar alat SWI. WI CV004 juga memakai oven 105 derajat C minimal 24 jam untuk bagian lab (tidak dimasukkan).</t>
         </is>
       </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="n"/>
+      <c r="H44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -1607,6 +1937,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="n"/>
+      <c r="H45" s="2" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -1634,6 +1971,13 @@
 2. Tambahan. Sumber menyebut standar ASTM tetapi tanpa volume isi, ayakan partikel kasar atau hasil detik per quart; hanya cek cepat, bukan kurva rheologi.</t>
         </is>
       </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="n"/>
+      <c r="H46" s="2" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -1659,6 +2003,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="n"/>
+      <c r="H47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -1688,6 +2039,13 @@
 3. Tambahan; rumus dosis terkonfirmasi (dosis x massa slurry x persen padatan / (kekuatan x 1.000.000)). Sumber tidak mencantumkan kontrol HCN padahal tailing bersianida; titik sampel dan pompa PU-372 milik Martabe.</t>
         </is>
       </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="n"/>
+      <c r="H48" s="2" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -1713,6 +2071,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="n"/>
+      <c r="H49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -1738,6 +2103,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="n"/>
+      <c r="H50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -1763,6 +2135,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="n"/>
+      <c r="H51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -1788,6 +2167,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="n"/>
+      <c r="H52" s="2" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -1813,6 +2199,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="n"/>
+      <c r="H53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -1838,6 +2231,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="n"/>
+      <c r="H54" s="2" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -1863,6 +2263,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="n"/>
+      <c r="H55" s="2" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -1888,6 +2295,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="n"/>
+      <c r="H56" s="2" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -1913,6 +2327,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="n"/>
+      <c r="H57" s="2" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">
@@ -1938,6 +2359,13 @@
           <t>SWI lebih lengkap dan dipertahankan. Dari Martabe hanya dua hal: cek buret digital terbaca 0.00 dan cek kedaluwarsa AgNO3. Titik akhir Martabe 'merah muda' tidak dipakai.</t>
         </is>
       </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="n"/>
+      <c r="H58" s="2" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n">
@@ -1965,6 +2393,13 @@
 2. Bertentangan: titik akhir 'soft pink' keliru (fenolftalein tidak berwarna pada titik akhir); SWI dipakai. Titran '5 persen' bukan molaritas, harus distandarisasi.</t>
         </is>
       </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="n"/>
+      <c r="H59" s="2" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -1990,6 +2425,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="n"/>
+      <c r="H60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2015,6 +2457,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="n"/>
+      <c r="H61" s="2" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2040,6 +2489,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="n"/>
+      <c r="H62" s="2" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -2069,6 +2525,13 @@
 3. Tambahan. V1.2 tidak punya langkah ulang dengan kaustik padahal tabelnya ada; satuan konsumsi mL/L untuk reagen padat; data berisi salah ketik. Satu penambahan 0.5 g melompatkan pH dari 6.2 ke 9.58 sehingga dosis perlu lebih kecil mendekati pH 7.</t>
         </is>
       </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="n"/>
+      <c r="H63" s="2" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -2094,6 +2557,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="n"/>
+      <c r="H64" s="2" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -2119,6 +2589,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="n"/>
+      <c r="H65" s="2" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -2144,6 +2621,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="n"/>
+      <c r="H66" s="2" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2169,6 +2653,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="n"/>
+      <c r="H67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2194,6 +2685,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="n"/>
+      <c r="H68" s="2" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -2225,6 +2723,13 @@
 4. Versi lebih awal dari uji adsorpsi slurry; tujuan H2SO4 5 persen dan 1 persen tidak dijelaskan.</t>
         </is>
       </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="n"/>
+      <c r="H69" s="2" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n">
@@ -2262,6 +2767,13 @@
 7. Tambahan. Kalibrasi memakai air; perlu konfirmasi pada laju uji (150 dan 300 mL/jam).</t>
         </is>
       </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="n"/>
+      <c r="H70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -2287,6 +2799,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="2" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -2312,6 +2831,13 @@
           <t>Martabe hanya langkah lime; tujuan menyebut peroxide tanpa dosis; pH awal dan kandungan sianida tidak disebut; PPE di bawah standar. Rute detox tidak tercakup.</t>
         </is>
       </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="n"/>
+      <c r="H72" s="2" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -2337,6 +2863,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="n"/>
+      <c r="H73" s="2" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -2362,6 +2895,13 @@
           <t>Bertentangan dengan Part A. Saya batasi ke indikator dan desikan saja, bukan standar atau sianida, dan perlu persetujuan kebijakan. Suhu oven tidak disebut.</t>
         </is>
       </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="n"/>
+      <c r="H74" s="2" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -2387,6 +2927,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="n"/>
+      <c r="H75" s="2" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -2412,6 +2959,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="n"/>
+      <c r="H76" s="2" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -2437,6 +2991,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="n"/>
+      <c r="H77" s="2" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -2462,6 +3023,13 @@
           <t>Tambahan ukur kuantitatif. Tidak ada nilai penerimaan dan cara merata-ratakan.</t>
         </is>
       </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="n"/>
+      <c r="H78" s="2" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -2487,6 +3055,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="n"/>
+      <c r="H79" s="2" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -2516,6 +3091,13 @@
 3. Bertentangan: tiga titik (SWI) vs dua titik; SWI dipertahankan kecuali dua titik disetujui. Martabe tidak mencatat slope dan offset.</t>
         </is>
       </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="n"/>
+      <c r="H80" s="2" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -2541,6 +3123,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="n"/>
+      <c r="H81" s="2" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -2566,6 +3155,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="n"/>
+      <c r="H82" s="2" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -2591,6 +3187,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="n"/>
+      <c r="H83" s="2" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -2616,6 +3219,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="n"/>
+      <c r="H84" s="2" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -2641,6 +3251,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="n"/>
+      <c r="H85" s="2" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -2666,6 +3283,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="n"/>
+      <c r="H86" s="2" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -2691,6 +3315,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="n"/>
+      <c r="H87" s="2" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -2716,6 +3347,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="n"/>
+      <c r="H88" s="2" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -2741,6 +3379,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="n"/>
+      <c r="H89" s="2" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -2766,6 +3411,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="n"/>
+      <c r="H90" s="2" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -2791,6 +3443,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="n"/>
+      <c r="H91" s="2" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -2816,6 +3475,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="n"/>
+      <c r="H92" s="2" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -2841,6 +3507,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="n"/>
+      <c r="H93" s="2" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -2866,6 +3539,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="n"/>
+      <c r="H94" s="2" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -2891,6 +3571,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="n"/>
+      <c r="H95" s="2" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">
@@ -2916,6 +3603,13 @@
           <t>Sumber meminta alarm HCN di bawah 10 ppm; SWI 5 ppm (diterapkan). Langkah mengacu foto yang tidak ikut; perangkat HCl Martabe belum tentu ada di Cynoprobe Anda. Operasi harian tidak tercakup.</t>
         </is>
       </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="n"/>
+      <c r="H96" s="2" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n">
@@ -2943,6 +3637,13 @@
 2. Standar detox tidak konsisten di sumber; perlu dipetakan ke analyser 051-CA-002.</t>
         </is>
       </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G97" s="5" t="n"/>
+      <c r="H97" s="2" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -2968,6 +3669,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F98" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G98" s="5" t="n"/>
+      <c r="H98" s="2" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -2993,6 +3701,13 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G99" s="5" t="n"/>
+      <c r="H99" s="2" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -3018,9 +3733,21 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="G100" s="5" t="n"/>
+      <c r="H100" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E100"/>
+  <autoFilter ref="A1:H100"/>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Sudah,Belum"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-002 and 201-003 to Heritage format; generalise builder
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -583,11 +583,19 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Dikonversi ke format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-002-003.md</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -615,11 +623,19 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Dikonversi ke format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-002-003.md</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-004 to Heritage format with carbon-in-launder check as Step 5
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -663,11 +663,19 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; carbon-in-launder (Martabe WI-00058) jadi Step 5, DRAFT; lihat docs/Format-Heritage/Catatan-Perubahan-201-004.md</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-005 to Heritage format with C2 check and calibration
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -705,11 +705,19 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; C2 check (Step 4) dan C2 calibration (Step 5) dari Martabe, DRAFT; lihat docs/Format-Heritage/Catatan-Perubahan-201-005.md</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-006 to 201-012 to Heritage format
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -745,11 +745,19 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -777,11 +785,19 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -809,11 +825,19 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -841,11 +865,19 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -873,11 +905,19 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -905,11 +945,19 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -937,11 +985,19 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-006-012.md</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-013 to Heritage format with approved Martabe Parts B, C, D
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1029,11 +1029,19 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; Part B, C, D Martabe disetujui dan dimasukkan (Step 3-5, DRAFT); lihat docs/Format-Heritage/Catatan-Perubahan-201-013.md</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-014 to 201-016 to Heritage format
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1069,11 +1069,19 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-014-016.md</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1101,11 +1109,19 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-014-016.md</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1133,11 +1149,19 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-014-016.md</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-017 and 201-020 to Heritage; move flocculant solution sampling to reagent SWI
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1189,11 +1189,19 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; flocculant solution sampling (Martabe WI-00064) dipindah ke 201-020 (area reagent); lihat docs/Format-Heritage/Catatan-Perubahan-201-017-020.md</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1289,11 +1297,19 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; Part B, C, D Martabe dan flocculant solution sampling (dari 201-017) sebagai Step 4-7, DRAFT; lihat docs/Format-Heritage/Catatan-Perubahan-201-017-020.md</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-018 to Heritage format
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1229,11 +1229,19 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-018.md</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-019 to Heritage format; replace NOT FOR USE with sampling-point update note
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1269,11 +1269,19 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; teknik sampling Martabe jadi Step 2-3; NOT FOR USE diganti catatan: titik sampling perlu diupdate; lihat docs/Format-Heritage/Catatan-Perubahan-201-019.md</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-201-021 to 201-025 to Heritage format; 201 series complete
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1353,11 +1353,19 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-021-025.md</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
@@ -1387,11 +1395,19 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-021-025.md; Part B dan C Martabe jadi Step 4-5, DRAFT</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1419,11 +1435,19 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-021-025.md</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1451,11 +1475,19 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-021-025.md</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1483,11 +1515,19 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-201-021-025.md</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-203 batch 1 (001, 004-009, 011, 012) to Heritage format
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1555,11 +1555,19 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
@@ -1651,11 +1659,19 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1683,11 +1699,19 @@
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1715,11 +1739,19 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1747,11 +1779,19 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1779,11 +1819,19 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1811,11 +1859,19 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
@@ -1875,11 +1931,19 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -1907,11 +1971,19 @@
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-203-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-203-002 and 203-003 to Heritage format (SWI cutter method only)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1595,11 +1595,19 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; metode Martabe (sampling manual) tidak dimasukkan karena SWI memakai cutter dengan pompa; lihat docs/Format-Heritage/Catatan-Perubahan-203-002-003.md</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
@@ -1627,11 +1635,19 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; metode Martabe (sampling manual) tidak dimasukkan karena SWI memakai cutter dengan pompa; lihat docs/Format-Heritage/Catatan-Perubahan-203-002-003.md</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-203-010 to Heritage (no shutdown intertank inspection); set 201-004 carbon-in-launder check to hourly
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -1915,11 +1915,19 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; Part B Martabe (angkat intertank screen saat shutdown) tidak dimasukkan: inspeksi perawatan, bukan pengecekan rutin; lihat docs/Format-Heritage/Catatan-Perubahan-203-010.md</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-204 batch 1 (16 SWI) to Heritage format; add 204 register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -2035,11 +2035,19 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2067,11 +2075,19 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2099,11 +2115,19 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md; tetap NOT FOR USE (laser sizer belum dibeli)</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2131,11 +2155,19 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2163,11 +2195,19 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n">
@@ -2227,11 +2267,19 @@
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G45" s="5" t="n"/>
-      <c r="H45" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n">
@@ -2293,11 +2341,19 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G47" s="5" t="n"/>
-      <c r="H47" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -2361,11 +2417,19 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G49" s="5" t="n"/>
-      <c r="H49" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2393,11 +2457,19 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="n"/>
-      <c r="H50" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2425,11 +2497,19 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G51" s="5" t="n"/>
-      <c r="H51" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2457,11 +2537,19 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G52" s="5" t="n"/>
-      <c r="H52" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2489,11 +2577,19 @@
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G53" s="5" t="n"/>
-      <c r="H53" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2521,11 +2617,19 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G54" s="5" t="n"/>
-      <c r="H54" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2553,11 +2657,19 @@
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G55" s="5" t="n"/>
-      <c r="H55" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2585,11 +2697,19 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G56" s="5" t="n"/>
-      <c r="H56" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2617,11 +2737,19 @@
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G57" s="5" t="n"/>
-      <c r="H57" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-204-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-207-001 to 207-006 (automatic samplers) to Heritage; add 207 register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -3853,11 +3853,19 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G90" s="5" t="n"/>
-      <c r="H90" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; tetap NOT FOR USE (desain sampler dan cutter belum ada); lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -3885,11 +3893,19 @@
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G91" s="5" t="n"/>
-      <c r="H91" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; tetap NOT FOR USE (desain sampler dan cutter belum ada); lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -3917,11 +3933,19 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G92" s="5" t="n"/>
-      <c r="H92" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; tetap NOT FOR USE (desain sampler dan cutter belum ada); lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -3949,11 +3973,19 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G93" s="5" t="n"/>
-      <c r="H93" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; tetap NOT FOR USE (desain sampler dan cutter belum ada); lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -3981,11 +4013,19 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G94" s="5" t="n"/>
-      <c r="H94" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; tetap NOT FOR USE (desain sampler dan cutter belum ada); lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
@@ -4013,11 +4053,19 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G95" s="5" t="n"/>
-      <c r="H95" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; lihat docs/Format-Heritage/Catatan-Perubahan-207-001-006.md</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-206 batch 1 (11 SWIs without Martabe additions) to Heritage; add 206 register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -3433,11 +3433,19 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G77" s="5" t="n"/>
-      <c r="H77" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n">
@@ -3497,11 +3505,19 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="n"/>
-      <c r="H79" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n">
@@ -3565,11 +3581,19 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="n"/>
-      <c r="H81" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -3597,11 +3621,19 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="n"/>
-      <c r="H82" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -3629,11 +3661,19 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G83" s="5" t="n"/>
-      <c r="H83" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -3661,11 +3701,19 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G84" s="5" t="n"/>
-      <c r="H84" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -3693,11 +3741,19 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G85" s="5" t="n"/>
-      <c r="H85" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; APD ditambah proteksi telinga (bench mill), sesuai persetujuan 204; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -3725,11 +3781,19 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="n"/>
-      <c r="H86" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -3757,11 +3821,19 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="n"/>
-      <c r="H87" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -3789,11 +3861,19 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G88" s="5" t="n"/>
-      <c r="H88" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -3821,11 +3901,19 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G89" s="5" t="n"/>
-      <c r="H89" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO210; lihat docs/Format-Heritage/Catatan-Perubahan-206-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">

</xml_diff>

<commit_message>
Convert SWI-PRO-MET-205 batch 1 (12 SWIs without Martabe additions) to Heritage; add 205 register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Tabel-SWI-vs-Martabe.xlsx
+++ b/docs/Tabel-SWI-vs-Martabe.xlsx
@@ -2867,11 +2867,19 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G60" s="5" t="n"/>
-      <c r="H60" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -2899,11 +2907,19 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G61" s="5" t="n"/>
-      <c r="H61" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2931,11 +2947,19 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G62" s="5" t="n"/>
-      <c r="H62" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n">
@@ -2999,11 +3023,19 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G64" s="5" t="n"/>
-      <c r="H64" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3031,11 +3063,19 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G65" s="5" t="n"/>
-      <c r="H65" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3063,11 +3103,19 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G66" s="5" t="n"/>
-      <c r="H66" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; safety-critical, kerja sianida tidak sendirian; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3095,11 +3143,19 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G67" s="5" t="n"/>
-      <c r="H67" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3127,11 +3183,19 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G68" s="5" t="n"/>
-      <c r="H68" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; APD ditambah pelindung telinga (hazard hearing damage, Ro-Tap); lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n">
@@ -3241,11 +3305,19 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G71" s="5" t="n"/>
-      <c r="H71" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; APD ditambah pelindung telinga (hazard hearing damage, Ro-Tap); lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n">
@@ -3305,11 +3377,19 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="n"/>
-      <c r="H73" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n">
@@ -3369,11 +3449,19 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G75" s="5" t="n"/>
-      <c r="H75" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3401,11 +3489,19 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="G76" s="5" t="n"/>
-      <c r="H76" s="2" t="n"/>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Format Heritage; isi SWI dipertahankan, tidak ada padanan Martabe; Parent procedure HM-PRC-VXX-PRO209; lihat docs/Format-Heritage/Catatan-Perubahan-205-batch1.md</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">

</xml_diff>